<commit_message>
Adicion de documentos para estimaciones
</commit_message>
<xml_diff>
--- a/Data anual/total_pred_final.xlsx
+++ b/Data anual/total_pred_final.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F427"/>
+  <dimension ref="A1:F451"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9832,6 +9832,390 @@
         <v>0.1963705429604246</v>
       </c>
     </row>
+    <row r="428">
+      <c r="A428" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>MONIQUIRA_BOYACA</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr"/>
+      <c r="D428" t="n">
+        <v>1.041926018843008</v>
+      </c>
+      <c r="E428" t="inlineStr"/>
+      <c r="F428" t="inlineStr"/>
+    </row>
+    <row r="429">
+      <c r="A429" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>SAN JOSE DE PARE_BOYACA</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr"/>
+      <c r="D429" t="n">
+        <v>0.996282595610221</v>
+      </c>
+      <c r="E429" t="inlineStr"/>
+      <c r="F429" t="inlineStr"/>
+    </row>
+    <row r="430">
+      <c r="A430" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>SANTANA_BOYACA</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr"/>
+      <c r="D430" t="n">
+        <v>0.8842662679763932</v>
+      </c>
+      <c r="E430" t="inlineStr"/>
+      <c r="F430" t="inlineStr"/>
+    </row>
+    <row r="431">
+      <c r="A431" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>TOGUI_BOYACA</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr"/>
+      <c r="D431" t="n">
+        <v>1.030123265829729</v>
+      </c>
+      <c r="E431" t="inlineStr"/>
+      <c r="F431" t="inlineStr"/>
+    </row>
+    <row r="432">
+      <c r="A432" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>AGUADA_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr"/>
+      <c r="D432" t="n">
+        <v>0.9527031356130036</v>
+      </c>
+      <c r="E432" t="inlineStr"/>
+      <c r="F432" t="inlineStr"/>
+    </row>
+    <row r="433">
+      <c r="A433" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>BARBOSA_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr"/>
+      <c r="D433" t="n">
+        <v>0.9571895821823624</v>
+      </c>
+      <c r="E433" t="inlineStr"/>
+      <c r="F433" t="inlineStr"/>
+    </row>
+    <row r="434">
+      <c r="A434" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>CHARALA_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr"/>
+      <c r="D434" t="n">
+        <v>1.127762839422976</v>
+      </c>
+      <c r="E434" t="inlineStr"/>
+      <c r="F434" t="inlineStr"/>
+    </row>
+    <row r="435">
+      <c r="A435" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>CHIPATA_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr"/>
+      <c r="D435" t="n">
+        <v>0.9750684428845017</v>
+      </c>
+      <c r="E435" t="inlineStr"/>
+      <c r="F435" t="inlineStr"/>
+    </row>
+    <row r="436">
+      <c r="A436" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>CONFINES_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr"/>
+      <c r="D436" t="n">
+        <v>0.9998836311003292</v>
+      </c>
+      <c r="E436" t="inlineStr"/>
+      <c r="F436" t="inlineStr"/>
+    </row>
+    <row r="437">
+      <c r="A437" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>CURITI_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr"/>
+      <c r="D437" t="n">
+        <v>1.099461023242466</v>
+      </c>
+      <c r="E437" t="inlineStr"/>
+      <c r="F437" t="inlineStr"/>
+    </row>
+    <row r="438">
+      <c r="A438" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>EL SOCORRO_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr"/>
+      <c r="D438" t="n">
+        <v>1.043786646650915</v>
+      </c>
+      <c r="E438" t="inlineStr"/>
+      <c r="F438" t="inlineStr"/>
+    </row>
+    <row r="439">
+      <c r="A439" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>GUADALUPE_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr"/>
+      <c r="D439" t="n">
+        <v>0.89820195268585</v>
+      </c>
+      <c r="E439" t="inlineStr"/>
+      <c r="F439" t="inlineStr"/>
+    </row>
+    <row r="440">
+      <c r="A440" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>GUAPOTA_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr"/>
+      <c r="D440" t="n">
+        <v>0.9299263884732939</v>
+      </c>
+      <c r="E440" t="inlineStr"/>
+      <c r="F440" t="inlineStr"/>
+    </row>
+    <row r="441">
+      <c r="A441" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>GUEPSA_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr"/>
+      <c r="D441" t="n">
+        <v>0.9816993493167159</v>
+      </c>
+      <c r="E441" t="inlineStr"/>
+      <c r="F441" t="inlineStr"/>
+    </row>
+    <row r="442">
+      <c r="A442" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>OCAMONTE_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr"/>
+      <c r="D442" t="n">
+        <v>0.8975606087466284</v>
+      </c>
+      <c r="E442" t="inlineStr"/>
+      <c r="F442" t="inlineStr"/>
+    </row>
+    <row r="443">
+      <c r="A443" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>OIBA_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr"/>
+      <c r="D443" t="n">
+        <v>0.9287273288970375</v>
+      </c>
+      <c r="E443" t="inlineStr"/>
+      <c r="F443" t="inlineStr"/>
+    </row>
+    <row r="444">
+      <c r="A444" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>PALMAS DEL SOCORRO_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr"/>
+      <c r="D444" t="n">
+        <v>0.939414545844624</v>
+      </c>
+      <c r="E444" t="inlineStr"/>
+      <c r="F444" t="inlineStr"/>
+    </row>
+    <row r="445">
+      <c r="A445" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>PARAMO_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr"/>
+      <c r="D445" t="n">
+        <v>1.058752608575698</v>
+      </c>
+      <c r="E445" t="inlineStr"/>
+      <c r="F445" t="inlineStr"/>
+    </row>
+    <row r="446">
+      <c r="A446" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>PINCHOTE_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr"/>
+      <c r="D446" t="n">
+        <v>1.010201229449918</v>
+      </c>
+      <c r="E446" t="inlineStr"/>
+      <c r="F446" t="inlineStr"/>
+    </row>
+    <row r="447">
+      <c r="A447" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>PUENTE NACIONAL_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr"/>
+      <c r="D447" t="n">
+        <v>0.9906827530174942</v>
+      </c>
+      <c r="E447" t="inlineStr"/>
+      <c r="F447" t="inlineStr"/>
+    </row>
+    <row r="448">
+      <c r="A448" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>SAN BENITO_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr"/>
+      <c r="D448" t="n">
+        <v>0.9754069179021368</v>
+      </c>
+      <c r="E448" t="inlineStr"/>
+      <c r="F448" t="inlineStr"/>
+    </row>
+    <row r="449">
+      <c r="A449" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>SAN GIL_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr"/>
+      <c r="D449" t="n">
+        <v>1.003904351590677</v>
+      </c>
+      <c r="E449" t="inlineStr"/>
+      <c r="F449" t="inlineStr"/>
+    </row>
+    <row r="450">
+      <c r="A450" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>SUAITA_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr"/>
+      <c r="D450" t="n">
+        <v>1.01946559856141</v>
+      </c>
+      <c r="E450" t="inlineStr"/>
+      <c r="F450" t="inlineStr"/>
+    </row>
+    <row r="451">
+      <c r="A451" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>VALLE DE SAN JOSE_SANTANDER</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr"/>
+      <c r="D451" t="n">
+        <v>0.9981323568075137</v>
+      </c>
+      <c r="E451" t="inlineStr"/>
+      <c r="F451" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>